<commit_message>
samples: update screenshots with new 2026-06-16 images
</commit_message>
<xml_diff>
--- a/samples/sample_jira_analysis_output.xlsx
+++ b/samples/sample_jira_analysis_output.xlsx
@@ -397,15 +397,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H10"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
-    <col min="3" max="3" width="28.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="28.83203125" customWidth="1"/>
-    <col min="7" max="7" width="65.83203125" customWidth="1"/>
+    <col min="3" max="3" width="42.83203125" customWidth="1"/>
+    <col min="4" max="4" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="28.83203125" customWidth="1"/>
+    <col min="8" max="8" width="65.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -416,116 +417,261 @@
         <v>Loại vấn đề</v>
       </c>
       <c r="C1" t="str">
+        <v>Vấn đề khách hàng</v>
+      </c>
+      <c r="D1" t="str">
         <v>Root Cause</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>SLA Status</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Ưu tiên</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Escalate đến</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Gợi ý xử lý CS</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ISSUE-40991</v>
+        <v>ISSUE-41046</v>
       </c>
       <c r="B2" t="str">
-        <v>Account_ChangeInfo</v>
+        <v>Lending_paylater</v>
       </c>
       <c r="C2" t="str">
+        <v>+ UserID: 200105000035207 + TransID: 260614001940325 GD TikTok Shop đã dc hoàn tiền thành công về TKTS Lotte nhưng trạng thái giao dịch đối tác PROCESSING, KH chưa nhận được hoàn lại hạn mức khả dụng =&gt; Nhờ team kiểm tra nguyên nhân và HXL giúp.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>External Factors</v>
+      </c>
+      <c r="E2" t="str">
+        <v>OK</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Không</v>
+      </c>
+      <c r="G2" t="str">
         <v/>
       </c>
-      <c r="D2" t="str">
-        <v>OK</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Không</v>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v>Hướng dẫn lại cho khách hàng về quy trình chụp ảnh XMCV, kiểm tra quyền truy cập camera và đảm bảo điều kiện ánh sáng rõ ràng. Không cần escalate vì lỗi thuộc nhóm hiểu nhầm của khách.</v>
+      <c r="H2" t="str">
+        <v>Thông báo KH hoàn tiền đã về tài khoản đối tác, hướng dẫn KH chờ hệ thống cập nhật trạng thái hoặc liên hệ TikTok Shop nếu cần hỗ trợ thêm.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ISSUE-40967</v>
+        <v>ISSUE-41042</v>
       </c>
       <c r="B3" t="str">
-        <v>Promotion campaign</v>
+        <v>Payment_Telco</v>
       </c>
       <c r="C3" t="str">
+        <v>- Mô tả lỗi: KH khiếu nại hiển thị tiêu đề là VTVgo Plus 30 ngày nhưng mô tả là thời hạn sử dụng VTVgo Plus trong vòng 7 ngày kể từ khi nhận được tài khoản. =&gt; nhờ team hỗ trợ kiểm tra nguyên nhân và hướng xử lý - Thời gian thực hiện: 15 Th06 2026 06</v>
+      </c>
+      <c r="D3" t="str">
+        <v>User misuderstanding</v>
+      </c>
+      <c r="E3" t="str">
+        <v>OK</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Không</v>
+      </c>
+      <c r="G3" t="str">
         <v/>
       </c>
-      <c r="D3" t="str">
-        <v>OK</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Không</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Team Cấu hình Khuyến mãi</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Liên hệ Team Cấu hình Khuyến mãi để rà soát lại quy tắc và cấu hình chương trình 2748. Yêu cầu xác nhận lỗi cấu hình đã được sửa và đảm bảo khách hàng nhận đủ thưởng theo cam kết.</v>
+      <c r="H3" t="str">
+        <v>Giải thích rõ cho KH về sự khác biệt giữa tiêu đề và mô tả thời hạn sử dụng sản phẩm VTVgo Plus, xác nhận KH đã hiểu đúng thông tin.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ISSUE-40959</v>
+        <v>ISSUE-41024</v>
       </c>
       <c r="B4" t="str">
-        <v>Lending_paylater</v>
+        <v>Promotion campaign</v>
       </c>
       <c r="C4" t="str">
+        <v xml:space="preserve">+ UserID: 241123001502277 + TransID: 260612002393348 - RewardCode: 3460 - DLS_260213_753 - Thứ 6 Không Tiền Mặt - Đi Buýt 0Đ - Thời gian: 15:38:09 ngày 12/06/2026 - Vấn đề của KH: kh khiếu nại không được miễn phí vé xe Bus và thứ sáu cs kiểm tra tnc </v>
+      </c>
+      <c r="D4" t="str">
+        <v>User need more Information</v>
+      </c>
+      <c r="E4" t="str">
+        <v>OK</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Không</v>
+      </c>
+      <c r="G4" t="str">
         <v/>
       </c>
-      <c r="D4" t="str">
-        <v>OK</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Không</v>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v>Giải thích lại cho khách hàng về quy tắc tính dư nợ theo kỳ và phân biệt rõ giữa giao dịch tháng cũ đã thanh toán với giao dịch mới phát sinh.</v>
+      <c r="H4" t="str">
+        <v>Cung cấp lại điều kiện áp dụng khuyến mãi cho KH (chỉ áp dụng appid 4058), hướng dẫn KH kiểm tra lại ứng dụng khi sử dụng.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ISSUE-40957</v>
+        <v>ISSUE-41021</v>
       </c>
       <c r="B5" t="str">
-        <v>Account_Login/Register</v>
+        <v>Promotion campaign</v>
       </c>
       <c r="C5" t="str">
+        <v>UID 251010000508699 TID 260514001665922 Tên chương trình ZFS_260401_119 Hoàn đến 100K khi gửi tiết kiệm lần đầu KH gửi tiền tiết kiệm, đã đáo hạn nhưng chưa nhận được vé thưởng xác nhận được hoàn tiền. =&gt; nhờ team hỗ trợ kiểm tra nguyên nhân và hướng</v>
+      </c>
+      <c r="D5" t="str">
+        <v>User misuderstanding</v>
+      </c>
+      <c r="E5" t="str">
+        <v>OK</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Không</v>
+      </c>
+      <c r="G5" t="str">
         <v/>
       </c>
-      <c r="D5" t="str">
-        <v>OK</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Không</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Team Tài khoản &amp; An toàn bảo mật</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Xác minh thông tin UID 260328000503716, liên hệ team phụ trách tài khoản để reset giới hạn OTP ngoại lệ cho KH do tình huống khẩn cấp thanh lý.</v>
+      <c r="H5" t="str">
+        <v>Hướng dẫn lại quy định nhận cashback sau khi đáo hạn gửi tiết kiệm, kiểm tra lại điều kiện chương trình ZFS_260401_119 cho KH.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ISSUE-41017</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Lending_paylater</v>
+      </c>
+      <c r="C6" t="str">
+        <v xml:space="preserve">+ UserID: 250112000009926 + TransID: 260613004220435 - 260613004204424 + Giao dịch TPE pending -998 + Mô tả: Tại sao tôi đã thanh toán trừ xu của tôi, mà tài khoản tôi vẫn chưa thanh toán ví trả sau??? Tôi nợ ví trả sau 5000đồng , Làm tôi thanh toán </v>
+      </c>
+      <c r="D6" t="str">
+        <v>External Factors</v>
+      </c>
+      <c r="E6" t="str">
+        <v>OK</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Không</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>Xác nhận lại trạng thái giao dịch với cổng thanh toán TPE, hướng dẫn KH theo dõi số dư xu và trạng thái nợ trả chậm.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ISSUE-41009</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Lending_installment</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Dear team USer thanh toán dư nợ tài khoản trả sau tuy nhiên tài khoản trả sau chưa được gạch nợ nhờ team kiểm tra UserID:230518004509696 TransID:260610001493954 Cám ơn ạ</v>
+      </c>
+      <c r="D7" t="str">
+        <v>External Factors</v>
+      </c>
+      <c r="E7" t="str">
+        <v>OK</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Không</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Team Đối tác</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Liên hệ đối tác CIMB để đối soát giao dịch thành công nhưng chưa gạch nợ. Thông báo KH đang phối hợp kiểm tra.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>ISSUE-41008</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Payment_Telco</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Vấn đề cần hỗ trợ: Hiện CS kiểm tra giao diện nạp data gói VTVgo Plus 30 ngày, ở ứng dụng Zalopay hiển thị phía ngoài gói 30 ngày với giá 20,000đ nhưng khi truy cập chi tiết gói thì hiển thị 7 ngày (ảnh đính kèm). CS kiểm tra trên CPStool cũng hiển t</v>
+      </c>
+      <c r="D8" t="str">
+        <v>User misuderstanding</v>
+      </c>
+      <c r="E8" t="str">
+        <v>OK</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Không</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>Kiểm tra thông tin hiển thị gói cước VTVgo. Nếu là hiểu lầm, hướng dẫn lại KH về quyền lợi và thời hạn gói.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ISSUE-41005</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Lending_cashloan</v>
+      </c>
+      <c r="C9" t="str">
+        <v>+ UserID: 251222000004941 Vấn đề: Khách hàng đăng ký vay tiền TNEX báo lỗi 'Có gì đó không đúng, vui lòng bấm 'Gửi lại mã để xác thực mà mới', Khách hàng bấm kg gửi mã mới vẫn báo lỗi như trên. &gt;&gt;&gt; Nhờ DEV hỗ trợ kiểm tra thêm nguyên nhân và HXL Cash</v>
+      </c>
+      <c r="D9" t="str">
+        <v>External Factors</v>
+      </c>
+      <c r="E9" t="str">
+        <v>OK</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Không</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Team Đối tác</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Liên hệ đối tác TNEX kiểm tra lỗi OTP xác thực khi đăng ký vay. Thông báo KH đang xử lý sự cố bên thứ ba.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>ISSUE-41004</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Payment_OnlineMerchant</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Dear Team, Nhờ team hủy giao dịch giúp khách hàng dịch vụ auto debit apple để CS hỗ trợ đóng tài khoản manual cho khách hàng UID: 250826005011770 SĐT Zalopay: 0355452655 Nhu cầu: Đóng tài khoản. Lý do: bỏ sim, muốn đóng để dùng lại Binding ID : 25100</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Others</v>
+      </c>
+      <c r="E10" t="str">
+        <v>OK</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Không</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Team Tài khoản</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Xác nhận hủy dịch vụ auto debit Apple. Phối hợp với team phụ trách để hỗ trợ đóng tài khoản manual cho KH.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>